<commit_message>
Updated Excel tabel with queries
</commit_message>
<xml_diff>
--- a/backend/queries_by_difficulty.xlsx
+++ b/backend/queries_by_difficulty.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10111"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\laure\OneDrive\Documents\University\8_Semester\BA\Covbot\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lstampfl/Dropbox/Mac/Documents/University/8_Semester/BA/Covbot/backend/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E881292-4699-4847-B2AA-332A9F645D90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A579850-4604-D148-B12C-E97A1BAECC5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" xr2:uid="{23BBDD8F-E7EB-45C8-AE03-40A229D24D6C}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{23BBDD8F-E7EB-45C8-AE03-40A229D24D6C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -627,13 +627,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{854A03FF-80A6-4AF0-8B30-213E9069B8D1}">
   <dimension ref="A1:J70"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="61.06640625" customWidth="1"/>
+    <col min="1" max="1" width="61" customWidth="1"/>
     <col min="10" max="10" width="140.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -644,7 +644,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -655,7 +655,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -663,7 +663,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
@@ -674,7 +674,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
@@ -682,7 +682,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>7</v>
       </c>
@@ -693,7 +693,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>8</v>
       </c>
@@ -704,7 +704,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>9</v>
       </c>
@@ -715,7 +715,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>10</v>
       </c>
@@ -726,7 +726,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>11</v>
       </c>
@@ -737,7 +737,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>14</v>
       </c>
@@ -748,7 +748,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>18</v>
       </c>
@@ -759,7 +759,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>19</v>
       </c>
@@ -767,7 +767,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>21</v>
       </c>
@@ -775,7 +775,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>22</v>
       </c>
@@ -786,7 +786,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>25</v>
       </c>
@@ -794,7 +794,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>26</v>
       </c>
@@ -802,7 +802,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>27</v>
       </c>
@@ -810,7 +810,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>28</v>
       </c>
@@ -821,7 +821,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>29</v>
       </c>
@@ -832,7 +832,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>30</v>
       </c>
@@ -840,7 +840,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>32</v>
       </c>
@@ -851,7 +851,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>33</v>
       </c>
@@ -862,24 +862,24 @@
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A24" t="s">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A24" s="1" t="s">
         <v>34</v>
       </c>
       <c r="J24" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A25" t="s">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A25" s="1" t="s">
         <v>35</v>
       </c>
       <c r="J25" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A26" t="s">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A26" s="1" t="s">
         <v>36</v>
       </c>
       <c r="I26">
@@ -889,8 +889,8 @@
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A27" t="s">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A27" s="1" t="s">
         <v>38</v>
       </c>
       <c r="I27">
@@ -900,8 +900,8 @@
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A28" t="s">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A28" s="1" t="s">
         <v>39</v>
       </c>
       <c r="I28">
@@ -911,7 +911,10 @@
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A29" s="1" t="s">
+        <v>40</v>
+      </c>
       <c r="I29">
         <v>1</v>
       </c>
@@ -919,7 +922,10 @@
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A30" s="1" t="s">
+        <v>41</v>
+      </c>
       <c r="I30">
         <v>1</v>
       </c>
@@ -927,7 +933,10 @@
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A31" s="1" t="s">
+        <v>47</v>
+      </c>
       <c r="I31">
         <v>1</v>
       </c>
@@ -935,17 +944,17 @@
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A32" t="s">
-        <v>40</v>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A32" s="1" t="s">
+        <v>48</v>
       </c>
       <c r="J32" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A33" t="s">
-        <v>41</v>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A33" s="1" t="s">
+        <v>49</v>
       </c>
       <c r="I33">
         <v>1</v>
@@ -954,9 +963,9 @@
         <v>32</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A34" t="s">
-        <v>47</v>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A34" s="1" t="s">
+        <v>50</v>
       </c>
       <c r="I34">
         <v>1</v>
@@ -965,9 +974,9 @@
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A35" t="s">
-        <v>48</v>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A35" s="1" t="s">
+        <v>51</v>
       </c>
       <c r="I35">
         <v>1</v>
@@ -976,9 +985,9 @@
         <v>34</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A36" t="s">
-        <v>49</v>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A36" s="1" t="s">
+        <v>52</v>
       </c>
       <c r="I36">
         <v>1</v>
@@ -987,9 +996,9 @@
         <v>35</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A37" t="s">
-        <v>50</v>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A37" s="1" t="s">
+        <v>53</v>
       </c>
       <c r="I37">
         <v>1</v>
@@ -998,18 +1007,12 @@
         <v>36</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A38" t="s">
-        <v>51</v>
-      </c>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
       <c r="J38" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A39" t="s">
-        <v>52</v>
-      </c>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
       <c r="I39">
         <v>1</v>
       </c>
@@ -1017,10 +1020,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A40" t="s">
-        <v>53</v>
-      </c>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
       <c r="I40">
         <v>1</v>
       </c>
@@ -1028,7 +1028,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>54</v>
       </c>
@@ -1039,7 +1039,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>55</v>
       </c>
@@ -1050,7 +1050,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>56</v>
       </c>
@@ -1058,7 +1058,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>58</v>
       </c>
@@ -1066,7 +1066,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>60</v>
       </c>
@@ -1074,7 +1074,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>65</v>
       </c>
@@ -1082,7 +1082,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>66</v>
       </c>
@@ -1090,7 +1090,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>68</v>
       </c>
@@ -1101,7 +1101,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>69</v>
       </c>
@@ -1112,7 +1112,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
       <c r="I50">
         <v>1</v>
       </c>
@@ -1120,7 +1120,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
       <c r="I51">
         <v>1</v>
       </c>
@@ -1128,7 +1128,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
       <c r="I52">
         <v>1</v>
       </c>
@@ -1136,7 +1136,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
       <c r="I53">
         <v>1</v>
       </c>
@@ -1144,7 +1144,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
       <c r="I54">
         <v>1</v>
       </c>
@@ -1152,7 +1152,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
       <c r="I55">
         <v>1</v>
       </c>
@@ -1160,7 +1160,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
       <c r="I56">
         <v>1</v>
       </c>
@@ -1168,7 +1168,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.2">
       <c r="I57">
         <v>1</v>
       </c>
@@ -1176,12 +1176,12 @@
         <v>56</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.2">
       <c r="J58" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.2">
       <c r="I59">
         <v>1</v>
       </c>
@@ -1189,12 +1189,12 @@
         <v>58</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.2">
       <c r="J60" s="2" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.2">
       <c r="I61">
         <v>1</v>
       </c>
@@ -1202,27 +1202,27 @@
         <v>60</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.2">
       <c r="J62" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.2">
       <c r="J63" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.2">
       <c r="J64" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="65" spans="9:10" x14ac:dyDescent="0.45">
+    <row r="65" spans="9:10" x14ac:dyDescent="0.2">
       <c r="J65" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="66" spans="9:10" x14ac:dyDescent="0.45">
+    <row r="66" spans="9:10" x14ac:dyDescent="0.2">
       <c r="I66">
         <v>1</v>
       </c>
@@ -1230,7 +1230,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="67" spans="9:10" x14ac:dyDescent="0.45">
+    <row r="67" spans="9:10" x14ac:dyDescent="0.2">
       <c r="I67">
         <v>1</v>
       </c>
@@ -1238,12 +1238,12 @@
         <v>66</v>
       </c>
     </row>
-    <row r="68" spans="9:10" x14ac:dyDescent="0.45">
+    <row r="68" spans="9:10" x14ac:dyDescent="0.2">
       <c r="J68" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="69" spans="9:10" x14ac:dyDescent="0.45">
+    <row r="69" spans="9:10" x14ac:dyDescent="0.2">
       <c r="I69">
         <v>1</v>
       </c>
@@ -1251,7 +1251,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="70" spans="9:10" x14ac:dyDescent="0.45">
+    <row r="70" spans="9:10" x14ac:dyDescent="0.2">
       <c r="I70">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
Updated query Excel file
</commit_message>
<xml_diff>
--- a/backend/queries_by_difficulty.xlsx
+++ b/backend/queries_by_difficulty.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lstampfl/Dropbox/Mac/Documents/University/8_Semester/BA/Covbot/backend/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4461D3B-8EB1-D242-9E33-B11EF4EE99F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC28D900-EDA2-934A-996A-160225F7F76E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{23BBDD8F-E7EB-45C8-AE03-40A229D24D6C}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="70">
   <si>
     <t>How many new cases have been reported in Austria today?</t>
   </si>
@@ -202,9 +202,6 @@
     <t>How many people are vaccinated?</t>
   </si>
   <si>
-    <t>How many people were vaccinated tody?</t>
-  </si>
-  <si>
     <t>How many corona cases got reported today?</t>
   </si>
   <si>
@@ -245,13 +242,16 @@
   </si>
   <si>
     <t>Could you tell me which how many new COVID cases were reported in Austria on 2nd February 2022?</t>
+  </si>
+  <si>
+    <t>How many people were vaccinated today?</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -273,8 +273,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF9C5700"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -291,6 +298,11 @@
         <fgColor rgb="FFFFC7CE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -301,19 +313,22 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="3"/>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="4">
     <cellStyle name="Bad" xfId="2" builtinId="27"/>
     <cellStyle name="Good" xfId="1" builtinId="26"/>
+    <cellStyle name="Neutral" xfId="3" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -944,11 +959,11 @@
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="J32" t="s">
+      <c r="J32" s="3" t="s">
         <v>31</v>
       </c>
     </row>
@@ -1008,11 +1023,17 @@
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A38" s="1" t="s">
+        <v>54</v>
+      </c>
       <c r="J38" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A39" s="1" t="s">
+        <v>69</v>
+      </c>
       <c r="I39">
         <v>1</v>
       </c>
@@ -1021,6 +1042,9 @@
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A40" s="1" t="s">
+        <v>55</v>
+      </c>
       <c r="I40">
         <v>1</v>
       </c>
@@ -1029,8 +1053,8 @@
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A41" t="s">
-        <v>54</v>
+      <c r="A41" s="1" t="s">
+        <v>59</v>
       </c>
       <c r="I41">
         <v>1</v>
@@ -1040,8 +1064,8 @@
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A42" t="s">
-        <v>55</v>
+      <c r="A42" s="1" t="s">
+        <v>64</v>
       </c>
       <c r="I42">
         <v>1</v>
@@ -1051,49 +1075,40 @@
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A43" t="s">
-        <v>56</v>
+      <c r="A43" s="1" t="s">
+        <v>67</v>
       </c>
       <c r="J43" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
-        <v>58</v>
+      <c r="A44" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J44" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A45" t="s">
-        <v>60</v>
+      <c r="A45" s="1" t="s">
+        <v>56</v>
       </c>
       <c r="J45" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A46" t="s">
-        <v>65</v>
-      </c>
-      <c r="J46" t="s">
+      <c r="J46" s="2" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A47" t="s">
-        <v>66</v>
-      </c>
       <c r="J47" s="2" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A48" t="s">
-        <v>68</v>
-      </c>
       <c r="I48">
         <v>1</v>
       </c>
@@ -1101,10 +1116,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
-        <v>69</v>
-      </c>
+    <row r="49" spans="9:10" x14ac:dyDescent="0.2">
       <c r="I49">
         <v>1</v>
       </c>
@@ -1112,7 +1124,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="50" spans="9:10" x14ac:dyDescent="0.2">
       <c r="I50">
         <v>1</v>
       </c>
@@ -1120,7 +1132,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="51" spans="9:10" x14ac:dyDescent="0.2">
       <c r="I51">
         <v>1</v>
       </c>
@@ -1128,7 +1140,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="52" spans="9:10" x14ac:dyDescent="0.2">
       <c r="I52">
         <v>1</v>
       </c>
@@ -1136,7 +1148,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="53" spans="9:10" x14ac:dyDescent="0.2">
       <c r="I53">
         <v>1</v>
       </c>
@@ -1144,7 +1156,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="54" spans="9:10" x14ac:dyDescent="0.2">
       <c r="I54">
         <v>1</v>
       </c>
@@ -1152,7 +1164,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="55" spans="9:10" x14ac:dyDescent="0.2">
       <c r="I55">
         <v>1</v>
       </c>
@@ -1160,66 +1172,63 @@
         <v>54</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="56" spans="9:10" x14ac:dyDescent="0.2">
       <c r="I56">
         <v>1</v>
       </c>
       <c r="J56" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="57" spans="9:10" x14ac:dyDescent="0.2">
+      <c r="I57">
+        <v>1</v>
+      </c>
+      <c r="J57" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="I57">
-        <v>1</v>
-      </c>
-      <c r="J57" t="s">
+    <row r="58" spans="9:10" x14ac:dyDescent="0.2">
+      <c r="J58" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="J58" t="s">
+    <row r="59" spans="9:10" x14ac:dyDescent="0.2">
+      <c r="J59" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="I59">
-        <v>1</v>
-      </c>
-      <c r="J59" t="s">
+    <row r="60" spans="9:10" x14ac:dyDescent="0.2">
+      <c r="J60" s="2" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="J60" s="2" t="s">
+    <row r="61" spans="9:10" x14ac:dyDescent="0.2">
+      <c r="I61">
+        <v>1</v>
+      </c>
+      <c r="J61" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="I61">
-        <v>1</v>
-      </c>
-      <c r="J61" t="s">
+    <row r="62" spans="9:10" x14ac:dyDescent="0.2">
+      <c r="J62" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="J62" t="s">
+    <row r="63" spans="9:10" x14ac:dyDescent="0.2">
+      <c r="J63" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="J63" t="s">
+    <row r="64" spans="9:10" x14ac:dyDescent="0.2">
+      <c r="J64" t="s">
         <v>62</v>
-      </c>
-    </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="J64" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="65" spans="9:10" x14ac:dyDescent="0.2">
       <c r="J65" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="66" spans="9:10" x14ac:dyDescent="0.2">
@@ -1227,20 +1236,17 @@
         <v>1</v>
       </c>
       <c r="J66" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="67" spans="9:10" x14ac:dyDescent="0.2">
+      <c r="J67" t="s">
         <v>65</v>
-      </c>
-    </row>
-    <row r="67" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I67">
-        <v>1</v>
-      </c>
-      <c r="J67" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="68" spans="9:10" x14ac:dyDescent="0.2">
       <c r="J68" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="69" spans="9:10" x14ac:dyDescent="0.2">
@@ -1248,7 +1254,7 @@
         <v>1</v>
       </c>
       <c r="J69" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="70" spans="9:10" x14ac:dyDescent="0.2">
@@ -1256,7 +1262,7 @@
         <v>1</v>
       </c>
       <c r="J70" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>